<commit_message>
Update submission files with final trained outputs and Kaggle link
</commit_message>
<xml_diff>
--- a/submissions/2A202602454_TranThanhThai/results.xlsx
+++ b/submissions/2A202602454_TranThanhThai/results.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Backbones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Training" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Inference" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Final" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="PerClass" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Latency" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Summary" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backbones" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Training" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inference" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PerClass" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latency" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,13 +23,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +43,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -48,12 +51,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,67 +435,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>exp_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>backbone</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>tag trọng số</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>#tham số (M)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>GMAC</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>độ phân giải</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>epoch</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>macro-F1 val</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>top-1 val</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>thời gian train/epoch (s)</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>độ trễ batch-1 (ms)</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>ghi chú</t>
         </is>
@@ -749,52 +761,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>exp_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>backbone</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>trục thay đổi (A–G)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>khác T00 ở điểm nào</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>macro-F1 val</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>top-1 val</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Δ so với T00</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>F1 các lớp hiếm (nếu có)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>ghi chú</t>
         </is>
@@ -1255,62 +1267,62 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>exp_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>phương pháp</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>mô hình/checkpoint dùng</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>K (số view hoặc số mô hình)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>macro-F1 val</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>top-1 val</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>ECE val</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>độ trễ p50 (ms) batch-1</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>độ trễ p95 (ms) batch-1</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>độ trễ p99 (ms) batch-1</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>thông lượng (ảnh/s)</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>chi phí tương đối so với I00</t>
         </is>
@@ -1595,42 +1607,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>exp_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>cấu hình (backbone + công thức + suy luận)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>macro-F1 val</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>macro-F1 test</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>top-1 test</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>ECE test</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>mean ± std qua seed (dòng tổng hợp)</t>
         </is>
@@ -1903,32 +1915,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>cấu hình</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>lớp</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>số ảnh test</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>precision</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>recall</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>F1</t>
         </is>
@@ -2381,47 +2393,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>cấu hình</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>GPU</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>dtype</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>batch</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>gộp BN (có/không)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>p50 (ms)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>p95 (ms)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>p99 (ms)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>ảnh/s</t>
         </is>
@@ -2664,47 +2676,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Hạng</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>exp_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cấu hình</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Macro-F1 Val</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Macro-F1 Test</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Top-1 Test</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>ECE Test</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Độ trễ p95 batch 1 (ms)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Đánh giá triển khai</t>
         </is>

</xml_diff>